<commit_message>
Mise a jour du 11-08-2026 16:42:19,02
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5682D52F-E570-4466-BBB2-09BAD370A03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65465AD0-199E-4E58-9F68-C95DC2E98480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
   <si>
     <t>n° Chapitre</t>
   </si>
@@ -124,6 +124,12 @@
   </si>
   <si>
     <t>Bidule</t>
+  </si>
+  <si>
+    <t>osJNKbrglyM</t>
+  </si>
+  <si>
+    <t>8RRnODCp9GE</t>
   </si>
 </sst>
 </file>
@@ -523,6 +529,9 @@
       <c r="H2" t="s">
         <v>15</v>
       </c>
+      <c r="J2" t="s">
+        <v>29</v>
+      </c>
       <c r="L2" t="s">
         <v>14</v>
       </c>
@@ -576,6 +585,9 @@
       <c r="D4" t="str">
         <f t="shared" si="0"/>
         <v>T.SF1.3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.4">
@@ -714,6 +726,12 @@
         <f>Liste!E4</f>
         <v>0</v>
       </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="str">

</xml_diff>

<commit_message>
Mise a jour du 13-08-2026 22:35:45,27
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liste" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plannification" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -46,10 +46,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,11 +396,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6"/>
   <cols>
-    <col width="9.765625" customWidth="1" style="1" min="4" max="4"/>
-    <col width="18" customWidth="1" style="1" min="5" max="5"/>
+    <col width="2.921875" customWidth="1" style="1" min="1" max="1"/>
+    <col width="4.61328125" customWidth="1" style="1" min="2" max="2"/>
+    <col width="4.4609375" customWidth="1" style="1" min="3" max="3"/>
+    <col width="3.15234375" customWidth="1" style="1" min="4" max="4"/>
+    <col width="44.07421875" customWidth="1" style="1" min="5" max="5"/>
+    <col width="3.3046875" customWidth="1" style="1" min="7" max="7"/>
+    <col width="3" customWidth="1" style="1" min="8" max="8"/>
+    <col width="2.3046875" customWidth="1" style="1" min="10" max="10"/>
+    <col width="2.23046875" customWidth="1" style="1" min="11" max="11"/>
+    <col width="1.921875" customWidth="1" style="1" min="13" max="13"/>
+    <col width="2.765625" customWidth="1" style="1" min="14" max="14"/>
+    <col width="2.3828125" customWidth="1" style="1" min="16" max="16"/>
+    <col width="2.3046875" customWidth="1" style="1" min="17" max="17"/>
+    <col width="2" customWidth="1" style="1" min="19" max="19"/>
+    <col width="2.23046875" customWidth="1" style="1" min="20" max="20"/>
+    <col width="18.23046875" customWidth="1" style="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,7 +524,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="29.15" customHeight="1" s="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>T</t>
@@ -526,48 +543,40 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiplier par 1 </t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>qrV9v5vRsz4</t>
+          <t>Demontrer une formule par récurrence</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>OIUi3MG8efY</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1900</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>9ALotzugzgQ</t>
+        <v>353</v>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>0vzO0zojbfI</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>3150</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>VNPOawm0RNg</t>
+        <v>583</v>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Y9p_V9ROp_A</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>706</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>qrV9v5vRsz4</t>
-        </is>
-      </c>
-      <c r="Q2" t="n">
-        <v>1900</v>
+        <v>647</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Revoir dérivé de x^n , e^x , ln(x), racine carré, 1/x</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Méthode 3 p 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="43.75" customHeight="1" s="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>T</t>
@@ -586,45 +595,40 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Diviser par 0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>AA9_JHSruJ0</t>
+          <t>Démontrer une inégalité par récurence</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>-v6seS__Hm0</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3153</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>qrV9v5vRsz4</t>
+        <v>413</v>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>ofPJoprpA2s</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>373</v>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>3eq423TrOoM</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>1900</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>qrV9v5vRsz4</t>
+        <v>398</v>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>_ez_5QZsVDM</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>1900</v>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>qrV9v5vRsz4</t>
-        </is>
-      </c>
-      <c r="T3" t="n">
-        <v>1900</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
+        <v>480</v>
       </c>
     </row>
     <row r="4">
@@ -634,33 +638,172 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>T.SF1.3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Calculer les termes d'une suite à la calculatrice</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Refaire exemple cours</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="29.15" customHeight="1" s="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>1</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>T.SF2.1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Diviser par 1</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>AA9_JHSruJ0</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>3153</v>
-      </c>
-    </row>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>T.SF1.4</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Déterminer le sens de variation d'une suite</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>DFz8LDKCw9Y</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>403</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>QRUbqrASmus</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>574</v>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>dPR3GyQycH0</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>344</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Méthode 1 p 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="29.15" customHeight="1" s="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>T.SF1.5</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Montrer qu'une suite est majorée, minorée ou bornée</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Dtp6URWws6s</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>554</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>TeRTbJxu25A</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>406</v>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>78LeZjY5MZw</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>729</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Méthode 2 p 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Etudier une suite à l'aide d'une fonction</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="H11" s="3" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -672,13 +815,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <cols>
     <col width="11.07421875" customWidth="1" style="1" min="1" max="1"/>
     <col width="13.15234375" customWidth="1" style="1" min="2" max="2"/>
-    <col width="11.07421875" customWidth="1" style="1" min="3" max="5"/>
-    <col width="11.07421875" customWidth="1" style="1" min="6" max="16384"/>
+    <col width="11.07421875" customWidth="1" style="1" min="3" max="7"/>
+    <col width="11.07421875" customWidth="1" style="1" min="8" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -774,9 +917,30 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T.SF3.1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Draw m life Terre</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T.SF1.5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Montrer qu'une suite est majorée, minorée ou bornée</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise a jour du 16-08-2026 22:42:30,40
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -396,7 +396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U178"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6"/>
   <cols>
     <col width="2.921875" customWidth="1" style="1" min="1" max="1"/>
@@ -407,7 +407,7 @@
     <col width="3.3046875" customWidth="1" style="1" min="7" max="7"/>
     <col width="7" customWidth="1" style="1" min="8" max="8"/>
     <col width="2.3046875" customWidth="1" style="1" min="10" max="10"/>
-    <col width="2.23046875" customWidth="1" style="1" min="11" max="11"/>
+    <col width="3.921875" customWidth="1" style="1" min="11" max="11"/>
     <col width="1.921875" customWidth="1" style="1" min="13" max="13"/>
     <col width="2.765625" customWidth="1" style="1" min="14" max="14"/>
     <col width="2.3828125" customWidth="1" style="1" min="16" max="16"/>
@@ -841,12 +841,1492 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
         <v>1</v>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>T.SF2.1</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Vecteur</t>
+        </is>
+      </c>
     </row>
     <row r="10"/>
-    <row r="11">
-      <c r="H11" s="3" t="n"/>
+    <row r="11" ht="29.15" customHeight="1" s="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>T.SF3.1</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conjecturer graphiquement la "convergence" ou "divergence" d'une suite </t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>0NBWe0RRjG4</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>591</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>BKt3SwTxykI</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="12" ht="29.15" customHeight="1" s="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>T.SF3.2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Additionner des limites</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>CEAbo1PoGl8</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="13" ht="29.15" customHeight="1" s="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>T.SF3.3</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Produit et Quotient de limite</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>FU5_5FDsoSw</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>561</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>OkpadGbc5zc</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="14" ht="29.15" customHeight="1" s="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>T.SF3.4</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Lever une indétermination en factorisant</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Gh8KXArr1hk</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>760</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>7rz7td0LZGY</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>223</v>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>jCFejEo2oQY</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="15" ht="29.15" customHeight="1" s="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>T.SF3.5</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Lever une indétermination avec des racines carrés</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>JbDvz3iobMk</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>275</v>
+      </c>
+      <c r="O15" s="3" t="n"/>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>HNxF6K5mvvk</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>T.SF3.6</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Utiliser le théorème de comparaison</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>7</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>T.SF3.7</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Utiliser le théorème d'encadrement (gendarmes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>T.SF3.8</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Justifier la convergence d'une suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="29.15" customHeight="1" s="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>9</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>T.SF3.9</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Limite d'une suite géométrique</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>oE7SS7T9PBM</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>434</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>MEp55lywR0M</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>274</v>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>HAcgnHFkVCc</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>470</v>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>kMelIoA4E2o</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>764</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Méthode 1p51</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" ht="43.75" customHeight="1" s="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>8</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>T.SF3.8</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>a recaser</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>ns-Hq9uVbS0</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -859,13 +2339,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <cols>
     <col width="11.07421875" customWidth="1" style="1" min="1" max="1"/>
     <col width="13.15234375" customWidth="1" style="1" min="2" max="2"/>
-    <col width="11.07421875" customWidth="1" style="1" min="3" max="9"/>
-    <col width="11.07421875" customWidth="1" style="1" min="10" max="16384"/>
+    <col width="11.07421875" customWidth="1" style="1" min="3" max="12"/>
+    <col width="11.07421875" customWidth="1" style="1" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1009,6 +2489,140 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T.SF2.1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Vecteur</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T.SF3.1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conjecturer graphiquement la "convergence" ou "divergence" d'une suite </t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>T.SF3.2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Additionner des limites</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>T.SF3.3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Produit et Quotient de limite</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>T.SF3.4</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lever une indétermination en factorisant</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>T.SF3.5</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lever une indétermination avec des racines carrés</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>T.SF3.6</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Utiliser le théorème de comparaison</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>T.SF3.7</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Utiliser le théorème d'encadrement (gendarmes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>T.SF3.8</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Justifier la convergence d'une suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>T.SF3.9</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Limite d'une suite géométrique</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>T.SF3.8</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>a recaser</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mise a jour du 30-08-2026 16:28:40,20
</commit_message>
<xml_diff>
--- a/contenu/Terminale.xlsx
+++ b/contenu/Terminale.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A80D28-B2FB-4BBF-A441-84EF2098A71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDFD1F58-C759-4578-8B28-6D3149ED26AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="14370" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -2850,7 +2850,7 @@
     </row>
     <row r="4" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
@@ -2862,7 +2862,7 @@
     </row>
     <row r="5" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
         <v>38</v>

</xml_diff>